<commit_message>
MJ: refresh lifetime report GHL codes with live pull (generated 479, redeemed 101)
</commit_message>
<xml_diff>
--- a/outputs/monkey-joes/MJ-Lifetime-Report.xlsx
+++ b/outputs/monkey-joes/MJ-Lifetime-Report.xlsx
@@ -829,7 +829,7 @@
   <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -838,7 +838,7 @@
     <row r="1">
       <c r="A1" s="36" t="inlineStr">
         <is>
-          <t>Monkey Joe's - Promo Codes: Generated &amp; Redeemed (lifetime, live from GHL)</t>
+          <t>Monkey Joe's - Promo Codes: Generated &amp; Redeemed (lifetime, live from GHL 2026-07-22)</t>
         </is>
       </c>
     </row>
@@ -878,13 +878,13 @@
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>158</v>
+        <v>219</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>236</v>
+        <v>260</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>394</v>
+        <v>479</v>
       </c>
     </row>
     <row r="6">
@@ -897,10 +897,10 @@
         <v>112</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7">
@@ -910,13 +910,13 @@
         </is>
       </c>
       <c r="B7" s="27" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8">
@@ -926,13 +926,13 @@
         </is>
       </c>
       <c r="B8" s="37" t="n">
-        <v>0.1645569620253164</v>
+        <v>0.1415525114155251</v>
       </c>
       <c r="C8" s="37" t="n">
-        <v>0.2796610169491525</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="D8" s="37" t="n">
-        <v>0.233502538071066</v>
+        <v>0.2108559498956159</v>
       </c>
     </row>
     <row r="10">
@@ -987,13 +987,13 @@
         </is>
       </c>
       <c r="B13" s="22" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C13" s="22" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D13" s="22" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14">
@@ -1035,13 +1035,13 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C16" s="27" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D16" s="27" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18">
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B20" s="22" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="B21" s="22" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22">
@@ -1100,27 +1100,27 @@
         </is>
       </c>
       <c r="B23" s="27" t="n">
-        <v>92</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Notes: 'Generated' = promo codes issued in GHL. 'Redeemed' = unique contacts with a redemption tag.</t>
+          <t>Notes: 'Generated' = promo codes issued in GHL. 'Redeemed' = unique contacts with a redemption tag (live count).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>66 redemptions are on older/manual contacts from before source-tagging; 26 carry a channel (FB 14 / Google 12).</t>
+          <t>66 redemptions are on older/manual contacts from before source-tagging; 35 carry a channel (FB 21 / Google 14).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Full in-store redemption count is also on William's verification page + Aluvii (BDAY25 parties).</t>
+          <t>Full in-store redemption count also lives on William's verification page; party bookings (BDAY25) in Aluvii.</t>
         </is>
       </c>
     </row>

</xml_diff>